<commit_message>
ajout slice typeDiplome au niveau de practitioner.qualification 3edc86e3a07fc0579949d09d53d6d7086dbeecf6
</commit_message>
<xml_diff>
--- a/ig/mc-deploy-1.0.0-ballot/StructureDefinition-as-dp-organization.xlsx
+++ b/ig/mc-deploy-1.0.0-ballot/StructureDefinition-as-dp-organization.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-05-26T16:24:55+00:00</t>
+    <t>2023-05-26T18:19:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -9640,7 +9640,7 @@
         <v>72</v>
       </c>
       <c r="G72" t="s" s="2">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H72" t="s" s="2">
         <v>71</v>
@@ -9744,7 +9744,7 @@
         <v>72</v>
       </c>
       <c r="G73" t="s" s="2">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H73" t="s" s="2">
         <v>71</v>
@@ -9848,7 +9848,7 @@
         <v>72</v>
       </c>
       <c r="G74" t="s" s="2">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H74" t="s" s="2">
         <v>71</v>

</xml_diff>